<commit_message>
Add pitch-deck details to CSAI data sheets
Enrich startup rows with product descriptions and websites from the Openwave
team pitch decks, add the Baku Metro Hackathon winner reported in a deck, and
note which decks could not be read.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rLvbjhK9XRJw9SDFpKNr8
</commit_message>
<xml_diff>
--- a/CSAI_2026_Governments_Data_Sheet_1_filled.xlsx
+++ b/CSAI_2026_Governments_Data_Sheet_1_filled.xlsx
@@ -2080,7 +2080,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="109" customHeight="1" s="39">
+    <row r="5" ht="139" customHeight="1" s="39">
       <c r="A5" s="61" t="inlineStr">
         <is>
           <t>Azerbaijan</t>
@@ -2093,7 +2093,7 @@
       </c>
       <c r="C5" s="61" t="inlineStr">
         <is>
-          <t>Participant registry and jury scoring sheet (Baku, 29–31 May 2026); no public URL in the materials</t>
+          <t>Participant registry, jury scoring sheet and team pitch decks (Baku, 29–31 May 2026). Initiator site cited in a participant deck: http://narimanov-ih.gov.az/az</t>
         </is>
       </c>
       <c r="D5" s="61" t="inlineStr">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="K5" s="61" t="inlineStr">
         <is>
-          <t>Challenges come from the public sector (government–startup) rather than corporations – verify it qualifies as corporate–startup stimulation. Narimanov is a district of Baku, so actual reach is district-level.</t>
+          <t>Challenges come from the public sector (government–startup) rather than corporations – verify it qualifies as corporate–startup stimulation. Narimanov is a district of Baku, so actual reach is district-level. Participant slides also show the Tedroid logo next to IDDA and the Narimanov executive authority – its role is not stated.</t>
         </is>
       </c>
     </row>
@@ -4993,7 +4993,7 @@
       </c>
       <c r="D5" s="62" t="inlineStr">
         <is>
-          <t>Digi Solution</t>
+          <t>Digi Solution (AI Detector)</t>
         </is>
       </c>
       <c r="E5" s="62" t="n"/>
@@ -5002,11 +5002,11 @@
       </c>
       <c r="G5" s="62" t="inlineStr">
         <is>
-          <t>Hackathon team (short activation, not a ≥8-week cohort). Winner. Rank 1 – 330 pts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="94" customHeight="1" s="39">
+          <t>Hackathon team (short activation, not a ≥8-week cohort). Winner. Rank 1 – 330 pts. Submission is a demo video ('DigiSolution AI Detector'); no slide deck.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="154" customHeight="1" s="39">
       <c r="A6" s="61" t="inlineStr">
         <is>
           <t>IDDA × Narimanov District Executive Authority</t>
@@ -5024,7 +5024,7 @@
       </c>
       <c r="D6" s="61" t="inlineStr">
         <is>
-          <t>ExaMinds</t>
+          <t>ExaMinds (Narimanov City Grind / AquaWatch)</t>
         </is>
       </c>
       <c r="E6" s="61" t="n"/>
@@ -5033,11 +5033,11 @@
       </c>
       <c r="G6" s="61" t="inlineStr">
         <is>
-          <t>Hackathon team (short activation, not a ≥8-week cohort). Winner. Rank 2 – 317 pts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="94" customHeight="1" s="39">
+          <t>Hackathon team (short activation, not a ≥8-week cohort). Winner. Rank 2 – 317 pts. Real-time district issue detection and response platform: citizen reporting with reward points, AI detection from bus/vehicle cameras (YOLO + VLM, trained on 50K+ road images) and AquaWatch flood-risk layer from satellite, terrain and rainfall data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="139" customHeight="1" s="39">
       <c r="A7" s="62" t="inlineStr">
         <is>
           <t>IDDA × Narimanov District Executive Authority</t>
@@ -5055,7 +5055,7 @@
       </c>
       <c r="D7" s="62" t="inlineStr">
         <is>
-          <t>Conflict</t>
+          <t>Conflict (Nərimanov+)</t>
         </is>
       </c>
       <c r="E7" s="62" t="n"/>
@@ -5064,11 +5064,11 @@
       </c>
       <c r="G7" s="62" t="inlineStr">
         <is>
-          <t>Hackathon team (short activation, not a ≥8-week cohort). Winner. Rank 3 – 302 pts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="94" customHeight="1" s="39">
+          <t>Hackathon team (short activation, not a ≥8-week cohort). Winner. Rank 3 – 302 pts. Platform that makes the city's hidden problems visible: photo, video and voice reports, AI issue detection, automatic assignment to the responsible agency and visual mapping. Model: B2B2G (300 AZN per building) and B2G.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="109" customHeight="1" s="39">
       <c r="A8" s="61" t="inlineStr">
         <is>
           <t>IDDA × Narimanov District Executive Authority</t>
@@ -5095,11 +5095,11 @@
       </c>
       <c r="G8" s="61" t="inlineStr">
         <is>
-          <t>Hackathon team (short activation, not a ≥8-week cohort). Rank 4 – 294 pts. MVP: https://nerve-city-nerve-pipe-monitoring-sy.vercel.app/</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="94" customHeight="1" s="39">
+          <t>Hackathon team (short activation, not a ≥8-week cohort). Rank 4 – 294 pts. MVP: https://nerve-city-nerve-pipe-monitoring-sy.vercel.app/ (pipe monitoring). Pitch deck is image-only, so its content could not be read.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="169" customHeight="1" s="39">
       <c r="A9" s="62" t="inlineStr">
         <is>
           <t>IDDA × Narimanov District Executive Authority</t>
@@ -5117,20 +5117,24 @@
       </c>
       <c r="D9" s="62" t="inlineStr">
         <is>
-          <t>Zəngəzur</t>
-        </is>
-      </c>
-      <c r="E9" s="62" t="n"/>
+          <t>Zəngəzur (HarAI)</t>
+        </is>
+      </c>
+      <c r="E9" s="62" t="inlineStr">
+        <is>
+          <t>https://zengezur2030.vercel.app/</t>
+        </is>
+      </c>
       <c r="F9" s="62" t="n">
         <v>2026</v>
       </c>
       <c r="G9" s="62" t="inlineStr">
         <is>
-          <t>Hackathon team (short activation, not a ≥8-week cohort). Rank 5 – 289 pts. MVP: https://zengezur2030.vercel.app/ ; Telegram bot t.me/zengezur_bot</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="94" customHeight="1" s="39">
+          <t>Hackathon team (short activation, not a ≥8-week cohort). Rank 5 – 289 pts. AI-based execution-control platform: a citizen photo becomes an AI-analysed 'Problem Passport' and an execution task closed with proof. B2G SaaS (pilot 30k–45k AZN + 3k–4k AZN/month); asks 30K AZN for a Narimanov pilot. Same team name as ZengezurBHOS (FinovateBank) and Zengezur BANM (WaterTech).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="124" customHeight="1" s="39">
       <c r="A10" s="61" t="inlineStr">
         <is>
           <t>IDDA × Narimanov District Executive Authority</t>
@@ -5148,7 +5152,7 @@
       </c>
       <c r="D10" s="61" t="inlineStr">
         <is>
-          <t>innohack</t>
+          <t>innohack (digitalNarimanov)</t>
         </is>
       </c>
       <c r="E10" s="61" t="n"/>
@@ -5157,11 +5161,11 @@
       </c>
       <c r="G10" s="61" t="inlineStr">
         <is>
-          <t>Hackathon team (short activation, not a ≥8-week cohort). Rank 6 – 286 pts. Working MVP (operator/admin/worker panels).</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="94" customHeight="1" s="39">
+          <t>Hackathon team (short activation, not a ≥8-week cohort). Rank 6 – 286 pts. Citizen mobile app for sending problems to the executive authority plus an AI-supported coordination platform (administrator/operator panels). Licence tiers from $3K to $250K+ per year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="139" customHeight="1" s="39">
       <c r="A11" s="62" t="inlineStr">
         <is>
           <t>IDDA × Narimanov District Executive Authority</t>
@@ -5179,7 +5183,7 @@
       </c>
       <c r="D11" s="62" t="inlineStr">
         <is>
-          <t>NAVI</t>
+          <t>NAVI (myCity)</t>
         </is>
       </c>
       <c r="E11" s="62" t="n"/>
@@ -5188,11 +5192,11 @@
       </c>
       <c r="G11" s="62" t="inlineStr">
         <is>
-          <t>Hackathon team (short activation, not a ≥8-week cohort). Rank 7 – 284 pts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="94" customHeight="1" s="39">
+          <t>Hackathon team (short activation, not a ≥8-week cohort). Rank 7 – 284 pts. Citizen–state mobile platform: AI photo and voice complaints, StreetBump road-defect detection from smartphone sensors, gamification points usable for public services. Same product owner as NAVI in the FinovateBank Hackathon.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="154" customHeight="1" s="39">
       <c r="A12" s="61" t="inlineStr">
         <is>
           <t>IDDA × Narimanov District Executive Authority</t>
@@ -5210,7 +5214,7 @@
       </c>
       <c r="D12" s="61" t="inlineStr">
         <is>
-          <t>Reacted</t>
+          <t>Reacted (NəzarətX)</t>
         </is>
       </c>
       <c r="E12" s="61" t="n"/>
@@ -5219,11 +5223,11 @@
       </c>
       <c r="G12" s="61" t="inlineStr">
         <is>
-          <t>Hackathon team (short activation, not a ≥8-week cohort). Rank 8 – 273 pts. MVP: https://nazaratx.netlify.app/</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="94" customHeight="1" s="39">
+          <t>Hackathon team (short activation, not a ≥8-week cohort). Rank 8 – 273 pts. MVP: https://nazaratx.netlify.app/. AI routes each complaint to the responsible agency and warns citizens about planned water/electricity outages; SaaS subscription and licences for district executive authorities, municipalities and utilities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="139" customHeight="1" s="39">
       <c r="A13" s="62" t="inlineStr">
         <is>
           <t>IDDA × Narimanov District Executive Authority</t>
@@ -5241,7 +5245,7 @@
       </c>
       <c r="D13" s="62" t="inlineStr">
         <is>
-          <t>NovaThink</t>
+          <t>NovaThink (AquaEye AI)</t>
         </is>
       </c>
       <c r="E13" s="62" t="n"/>
@@ -5250,11 +5254,11 @@
       </c>
       <c r="G13" s="62" t="inlineStr">
         <is>
-          <t>Hackathon team (short activation, not a ≥8-week cohort). Rank 9 – 270 pts. MVP: https://aquaeye-ai-baku.netlify.app</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="94" customHeight="1" s="39">
+          <t>Hackathon team (short activation, not a ≥8-week cohort). Rank 9 – 270 pts. MVP: https://aquaeye-ai-baku.netlify.app. Turns existing CCTV cameras into real-time flood sensors (YOLOv8-seg water segmentation, depth estimate, automatic alerts); B2G SaaS, target clients FHN, AYNA and municipalities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="139" customHeight="1" s="39">
       <c r="A14" s="61" t="inlineStr">
         <is>
           <t>IDDA × Narimanov District Executive Authority</t>
@@ -5272,7 +5276,7 @@
       </c>
       <c r="D14" s="61" t="inlineStr">
         <is>
-          <t>Super Tələbə</t>
+          <t>Super Tələbə (TəmizAI)</t>
         </is>
       </c>
       <c r="E14" s="61" t="n"/>
@@ -5281,11 +5285,11 @@
       </c>
       <c r="G14" s="61" t="inlineStr">
         <is>
-          <t>Hackathon team (short activation, not a ≥8-week cohort). Rank 10 – 269 pts. MVP: https://temizeka-swart.vercel.app/</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="94" customHeight="1" s="39">
+          <t>Hackathon team (short activation, not a ≥8-week cohort). Rank 10 – 269 pts. Demo: https://temizeka-swart.vercel.app/. AI app monitoring waste-container problems, built on Narimanov executive authority data; 85% model accuracy; 12-month plan from a 3-street pilot to the whole district.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="124" customHeight="1" s="39">
       <c r="A15" s="62" t="inlineStr">
         <is>
           <t>IDDA × Narimanov District Executive Authority</t>
@@ -5312,11 +5316,11 @@
       </c>
       <c r="G15" s="62" t="inlineStr">
         <is>
-          <t>Hackathon team (short activation, not a ≥8-week cohort). Rank 11 – 268 pts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="94" customHeight="1" s="39">
+          <t>Hackathon team (short activation, not a ≥8-week cohort). Rank 11 – 268 pts. Area-monitoring and automated coordination platform: dashboard, mobile app, tracking of responsible staff, status and deadlines. One-time platform licence for local government; free for citizens.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="109" customHeight="1" s="39">
       <c r="A16" s="61" t="inlineStr">
         <is>
           <t>IDDA × Narimanov District Executive Authority</t>
@@ -5334,7 +5338,7 @@
       </c>
       <c r="D16" s="61" t="inlineStr">
         <is>
-          <t>CoreApex</t>
+          <t>CoreApex (Mobilİcra)</t>
         </is>
       </c>
       <c r="E16" s="61" t="n"/>
@@ -5343,11 +5347,11 @@
       </c>
       <c r="G16" s="61" t="inlineStr">
         <is>
-          <t>Hackathon team (short activation, not a ≥8-week cohort). Rank 12 – 260 pts. MVP deployed on Vercel.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="94" customHeight="1" s="39">
+          <t>Hackathon team (short activation, not a ≥8-week cohort). Rank 12 – 260 pts. Digital coordination and execution platform: single request panel, inter-agency request flow, SLA/deadline escalation, live map with heatmap and simulation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="109" customHeight="1" s="39">
       <c r="A17" s="62" t="inlineStr">
         <is>
           <t>IDDA × Narimanov District Executive Authority</t>
@@ -5365,7 +5369,7 @@
       </c>
       <c r="D17" s="62" t="inlineStr">
         <is>
-          <t>WaveX</t>
+          <t>WaveX (myRegion)</t>
         </is>
       </c>
       <c r="E17" s="62" t="n"/>
@@ -5374,11 +5378,11 @@
       </c>
       <c r="G17" s="62" t="inlineStr">
         <is>
-          <t>Hackathon team (short activation, not a ≥8-week cohort). Rank 13 – 256 pts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="94" customHeight="1" s="39">
+          <t>Hackathon team (short activation, not a ≥8-week cohort). Rank 13 – 256 pts. 'See it, snap it, track it' reporting app: duplicate reports grouped into threads, AI moderation, coin rewards, hardware module and admin dashboard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="109" customHeight="1" s="39">
       <c r="A18" s="61" t="inlineStr">
         <is>
           <t>IDDA × Narimanov District Executive Authority</t>
@@ -5396,7 +5400,7 @@
       </c>
       <c r="D18" s="61" t="inlineStr">
         <is>
-          <t>CityFix</t>
+          <t>CityFix (DARGAH)</t>
         </is>
       </c>
       <c r="E18" s="61" t="n"/>
@@ -5405,11 +5409,11 @@
       </c>
       <c r="G18" s="61" t="inlineStr">
         <is>
-          <t>Hackathon team (short activation, not a ≥8-week cohort). Rank 14 – 250 pts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="94" customHeight="1" s="39">
+          <t>Hackathon team (short activation, not a ≥8-week cohort). Rank 14 – 250 pts. AI monitoring and service platform working through WhatsApp, Telegram and web chatbots (Next.js, FastAPI, Supabase); claims to cut operator workload by 80%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="124" customHeight="1" s="39">
       <c r="A19" s="62" t="inlineStr">
         <is>
           <t>IDDA × Narimanov District Executive Authority</t>
@@ -5436,7 +5440,7 @@
       </c>
       <c r="G19" s="62" t="inlineStr">
         <is>
-          <t>Hackathon team (short activation, not a ≥8-week cohort). Rank 15 – 234 pts.</t>
+          <t>Hackathon team (short activation, not a ≥8-week cohort). Rank 15 – 234 pts. Digital twin of Narimanov district: citizen reporting, central management panel, IDDA digital document-flow (RSD) integration and AI satellite-image analysis to detect illegal buildings.</t>
         </is>
       </c>
     </row>
@@ -5781,7 +5785,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="124" customHeight="1" s="39">
+    <row r="31" ht="154" customHeight="1" s="39">
       <c r="A31" s="62" t="inlineStr">
         <is>
           <t>ADSEA × SUP.VC</t>
@@ -5812,7 +5816,7 @@
       </c>
       <c r="G31" s="62" t="inlineStr">
         <is>
-          <t>Bootcamp/hackathon team (short activation, not a ≥8-week cohort). Sensor-based real-time water-quality monitoring (EC, nitrate, pH) for irrigation with AI analysis, crop-specific advice and a chatbot; main target market: Water Users' Associations.</t>
+          <t>Bootcamp/hackathon team (short activation, not a ≥8-week cohort). Sensor-based real-time water-quality monitoring (EC, nitrate, pH) for irrigation with AI analysis, crop-specific advice and a chatbot; main target market: Water Users' Associations. Team member Gudrat Abbasli also appears on the Zəngəzur team slide (Openwave).</t>
         </is>
       </c>
     </row>
@@ -5878,7 +5882,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="124" customHeight="1" s="39">
+    <row r="34" ht="154" customHeight="1" s="39">
       <c r="A34" s="61" t="inlineStr">
         <is>
           <t>ADSEA × SUP.VC</t>
@@ -5905,7 +5909,7 @@
       </c>
       <c r="G34" s="61" t="inlineStr">
         <is>
-          <t>Bootcamp/hackathon team (short activation, not a ≥8-week cohort). Data platform forecasting drainage/flood risk on farmland, with automated alerts, decision dashboards and an Azerbaijani-language AI chatbot; B2B (cooperatives) and B2C (farmers).</t>
+          <t>Bootcamp/hackathon team (short activation, not a ≥8-week cohort). Data platform forecasting drainage/flood risk on farmland, with automated alerts, decision dashboards and an Azerbaijani-language AI chatbot; B2B (cooperatives) and B2C (farmers). Team member Əvəz Əsgərov also appears on the Zəngəzur team slide (Openwave).</t>
         </is>
       </c>
     </row>
@@ -6037,7 +6041,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="109" customHeight="1" s="39">
+    <row r="39" ht="154" customHeight="1" s="39">
       <c r="A39" s="62" t="inlineStr">
         <is>
           <t>ADSEA × SUP.VC</t>
@@ -6064,7 +6068,7 @@
       </c>
       <c r="G39" s="62" t="inlineStr">
         <is>
-          <t>Bootcamp/hackathon team (short activation, not a ≥8-week cohort). AI-based differential water-tariff system: personalised monthly household limits by family profile, higher tariff and staged pressure reduction above the limit (B2G2C).</t>
+          <t>Bootcamp/hackathon team (short activation, not a ≥8-week cohort). AI-based differential water-tariff system: personalised monthly household limits by family profile, higher tariff and staged pressure reduction above the limit (B2G2C). Deck title slide names the Water and Melioration Scientific Research Institute.</t>
         </is>
       </c>
     </row>
@@ -6192,8 +6196,34 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="15.75" customHeight="1" s="39">
-      <c r="C44" s="36" t="n"/>
+    <row r="44" ht="94" customHeight="1" s="39">
+      <c r="A44" s="61" t="inlineStr">
+        <is>
+          <t>Baku Metropolitan CJSC (Baku Metro)</t>
+        </is>
+      </c>
+      <c r="B44" s="61" t="inlineStr">
+        <is>
+          <t>Baku Metro Hackathon</t>
+        </is>
+      </c>
+      <c r="C44" s="61" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D44" s="61" t="inlineStr">
+        <is>
+          <t>Zəngəzur</t>
+        </is>
+      </c>
+      <c r="E44" s="61" t="n"/>
+      <c r="F44" s="61" t="n"/>
+      <c r="G44" s="61" t="inlineStr">
+        <is>
+          <t>Hackathon team (short activation, not a ≥8-week cohort). 'Metro Hakaton 1-ci yer' (1st place) is listed on the team slide of Zəngəzur's Openwave pitch deck – self-reported; year not stated.</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="15.75" customHeight="1" s="39"/>
     <row r="46" ht="15.75" customHeight="1" s="39"/>

</xml_diff>